<commit_message>
Trim spreadsheet: drop GPA column, use avg net price, shrink headers
- Removed weighted-GPA-on-100 column (not published by these schools).
- Replaced the 00k+ column with the school's overall average net price.
- Smaller header font (9pt) and tightened column widths so the full table
  fits with minimal horizontal scrolling.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CUhjAk7h6xF2a3djroFRRG
</commit_message>
<xml_diff>
--- a/college_research.xlsx
+++ b/college_research.xlsx
@@ -32,11 +32,11 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -71,19 +71,19 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -450,80 +450,74 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="41" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="23" customWidth="1" min="10" max="10"/>
-    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="60" customHeight="1">
+    <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>School Name</t>
+          <t>School</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Location (City, State)</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Total Sticker Price / Year (Tuition + Fees + R&amp;B, no aid) [USD]</t>
+          <t>Sticker Price / Yr</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Avg Price Paid, Families $300k+ Income (or overall avg net price if unpublished)</t>
+          <t>Avg Net Price Paid</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Median SAT (Admitted Students)</t>
+          <t>Median SAT</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Median Weighted GPA (out of 100)</t>
+          <t>Accept Rate</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Acceptance Rate (%)</t>
+          <t>Applicants (2026)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Applicants (2026 cycle)</t>
+          <t>Admitted (2026)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Admitted (2026 cycle)</t>
+          <t>Enrolled (2026)</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Enrolled (2026 cycle)</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
           <t>Notes / Cycle Used</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Clemson University</t>
@@ -537,38 +531,31 @@
       <c r="C2" s="3" t="n">
         <v>52206</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Not published for $300k+; overall avg net price ~$25,700 used</t>
-        </is>
+      <c r="D2" s="3" t="n">
+        <v>25700</v>
       </c>
       <c r="E2" s="4" t="n">
         <v>1325</v>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Not published on 100 scale</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="n">
+      <c r="F2" s="5" t="n">
         <v>0.383</v>
       </c>
+      <c r="G2" s="6" t="n">
+        <v>61517</v>
+      </c>
       <c r="H2" s="6" t="n">
-        <v>61517</v>
+        <v>23586</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>23586</v>
-      </c>
-      <c r="J2" s="6" t="n">
         <v>4326</v>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024 cycle); 2026 cycle data not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="42" customHeight="1">
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Florida Atlantic University</t>
@@ -582,38 +569,31 @@
       <c r="C3" s="3" t="n">
         <v>42382</v>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Not published for $300k+; overall avg net price ~$13,600 used</t>
-        </is>
+      <c r="D3" s="3" t="n">
+        <v>13600</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>1120</v>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Not published on 100 scale</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="n">
+      <c r="F3" s="5" t="n">
         <v>0.6613</v>
       </c>
+      <c r="G3" s="6" t="n">
+        <v>31511</v>
+      </c>
       <c r="H3" s="6" t="n">
-        <v>31511</v>
+        <v>20838</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>20838</v>
-      </c>
-      <c r="J3" s="6" t="n">
         <v>4900</v>
       </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024 cycle); 2026 cycle data not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="42" customHeight="1">
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Florida State University</t>
@@ -627,38 +607,31 @@
       <c r="C4" s="3" t="n">
         <v>41427</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Not published for $300k+; overall avg net price ~$14,600 used</t>
-        </is>
+      <c r="D4" s="3" t="n">
+        <v>14600</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>1350</v>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Not published on 100 scale</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="n">
+      <c r="F4" s="5" t="n">
         <v>0.2422</v>
       </c>
+      <c r="G4" s="6" t="n">
+        <v>78272</v>
+      </c>
       <c r="H4" s="6" t="n">
-        <v>78272</v>
+        <v>18954</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>18954</v>
-      </c>
-      <c r="J4" s="6" t="n">
         <v>6800</v>
       </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024 cycle); 2026 cycle data not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="42" customHeight="1">
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>NC State University</t>
@@ -672,41 +645,34 @@
       <c r="C5" s="3" t="n">
         <v>51285</v>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Not published for $300k+; overall avg net price ~$16,900 used</t>
-        </is>
+      <c r="D5" s="3" t="n">
+        <v>16900</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>1370</v>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Not published on 100 scale</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="n">
+      <c r="F5" s="5" t="n">
         <v>0.417</v>
       </c>
+      <c r="G5" s="6" t="n">
+        <v>44043</v>
+      </c>
       <c r="H5" s="6" t="n">
-        <v>44043</v>
+        <v>18381</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>18381</v>
-      </c>
-      <c r="J5" s="6" t="n">
         <v>5412</v>
       </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024 cycle); 2026 cycle data not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Penn State University (University Park)</t>
+          <t>Penn State (University Park)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -717,38 +683,31 @@
       <c r="C6" s="3" t="n">
         <v>63284</v>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Not published for $300k+; overall avg net price ~$29,200 used</t>
-        </is>
+      <c r="D6" s="3" t="n">
+        <v>29200</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>1330</v>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Not published on 100 scale</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="n">
+      <c r="F6" s="5" t="n">
         <v>0.6056</v>
       </c>
+      <c r="G6" s="6" t="n">
+        <v>88478</v>
+      </c>
       <c r="H6" s="6" t="n">
-        <v>88478</v>
+        <v>53579</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>53579</v>
-      </c>
-      <c r="J6" s="6" t="n">
         <v>9800</v>
       </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024 cycle); 2026 cycle data not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1">
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Syracuse University</t>
@@ -762,38 +721,31 @@
       <c r="C7" s="3" t="n">
         <v>87840</v>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Not published for $300k+; overall avg net price ~$48,215 used</t>
-        </is>
+      <c r="D7" s="3" t="n">
+        <v>48215</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>1360</v>
       </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Not published on 100 scale</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n">
+      <c r="F7" s="5" t="n">
         <v>0.4592</v>
       </c>
+      <c r="G7" s="6" t="n">
+        <v>44480</v>
+      </c>
       <c r="H7" s="6" t="n">
-        <v>44480</v>
+        <v>20427</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>20427</v>
-      </c>
-      <c r="J7" s="6" t="n">
         <v>3835</v>
       </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024 cycle); 2026 cycle data not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1">
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>University of Alabama</t>
@@ -807,38 +759,31 @@
       <c r="C8" s="3" t="n">
         <v>55916</v>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Not published for $300k+; overall avg net price ~$26,900 used (IPEDS)</t>
-        </is>
+      <c r="D8" s="3" t="n">
+        <v>26900</v>
       </c>
       <c r="E8" s="4" t="n">
         <v>1290</v>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Not published on 100 scale (CDS reports ~3.76 unweighted / 4.0)</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="n">
+      <c r="F8" s="5" t="n">
         <v>0.7659999999999999</v>
       </c>
+      <c r="G8" s="6" t="n">
+        <v>56795</v>
+      </c>
       <c r="H8" s="6" t="n">
-        <v>56795</v>
+        <v>43531</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>43531</v>
-      </c>
-      <c r="J8" s="6" t="n">
         <v>8039</v>
       </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024 cycle); 2026 cycle data not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1">
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>University of Connecticut</t>
@@ -852,38 +797,31 @@
       <c r="C9" s="3" t="n">
         <v>58780</v>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Not published for $300k+; overall avg net price ~$23,800 used</t>
-        </is>
+      <c r="D9" s="3" t="n">
+        <v>23800</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>1340</v>
       </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Not published on 100 scale</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n">
+      <c r="F9" s="5" t="n">
         <v>0.5239</v>
       </c>
+      <c r="G9" s="6" t="n">
+        <v>55479</v>
+      </c>
       <c r="H9" s="6" t="n">
-        <v>55479</v>
+        <v>29065</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>29065</v>
-      </c>
-      <c r="J9" s="6" t="n">
         <v>3800</v>
       </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024 cycle); 2026 cycle data not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="42" customHeight="1">
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>University of Delaware</t>
@@ -897,38 +835,31 @@
       <c r="C10" s="3" t="n">
         <v>56090</v>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Not published for $300k+; overall avg net price ~$24,500 used</t>
-        </is>
+      <c r="D10" s="3" t="n">
+        <v>24500</v>
       </c>
       <c r="E10" s="4" t="n">
         <v>1295</v>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Not published on 100 scale</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="n">
+      <c r="F10" s="5" t="n">
         <v>0.706</v>
       </c>
+      <c r="G10" s="6" t="n">
+        <v>39995</v>
+      </c>
       <c r="H10" s="6" t="n">
-        <v>39995</v>
+        <v>28238</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>28238</v>
-      </c>
-      <c r="J10" s="6" t="n">
         <v>4400</v>
       </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024 cycle); 2026 cycle data not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="42" customHeight="1">
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>University of Louisville</t>
@@ -942,38 +873,31 @@
       <c r="C11" s="3" t="n">
         <v>44500</v>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Not published for $300k+; overall avg net price ~$19,785 used</t>
-        </is>
+      <c r="D11" s="3" t="n">
+        <v>19785</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>1150</v>
       </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Not published on 100 scale</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="n">
+      <c r="F11" s="5" t="n">
         <v>0.7940999999999999</v>
       </c>
+      <c r="G11" s="6" t="n">
+        <v>15668</v>
+      </c>
       <c r="H11" s="6" t="n">
-        <v>15668</v>
+        <v>12442</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>12442</v>
-      </c>
-      <c r="J11" s="6" t="n">
         <v>2900</v>
       </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024 cycle); 2026 cycle data not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="42" customHeight="1">
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>University of Miami</t>
@@ -987,38 +911,31 @@
       <c r="C12" s="3" t="n">
         <v>93892</v>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Not published for $300k+; overall avg net price ~$44,600 used</t>
-        </is>
+      <c r="D12" s="3" t="n">
+        <v>44600</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>1400</v>
       </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Not published on 100 scale</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="n">
+      <c r="F12" s="5" t="n">
         <v>0.189</v>
       </c>
+      <c r="G12" s="6" t="n">
+        <v>53954</v>
+      </c>
       <c r="H12" s="6" t="n">
-        <v>53954</v>
+        <v>10195</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>10195</v>
-      </c>
-      <c r="J12" s="6" t="n">
         <v>2400</v>
       </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024 cycle); 2026 cycle data not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="42" customHeight="1">
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>University of Pittsburgh</t>
@@ -1032,38 +949,31 @@
       <c r="C13" s="3" t="n">
         <v>60310</v>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Not published for $300k+; overall avg net price ~$27,400 used</t>
-        </is>
+      <c r="D13" s="3" t="n">
+        <v>27400</v>
       </c>
       <c r="E13" s="4" t="n">
         <v>1360</v>
       </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Not published on 100 scale</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="n">
+      <c r="F13" s="5" t="n">
         <v>0.5808</v>
       </c>
+      <c r="G13" s="6" t="n">
+        <v>60898</v>
+      </c>
       <c r="H13" s="6" t="n">
-        <v>60898</v>
+        <v>35372</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>35372</v>
-      </c>
-      <c r="J13" s="6" t="n">
         <v>4596</v>
       </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024 cycle); 2026 cycle data not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="42" customHeight="1">
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>University of Richmond</t>
@@ -1077,38 +987,31 @@
       <c r="C14" s="3" t="n">
         <v>84930</v>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Not published for $300k+; overall avg net price ~$32,700 used</t>
-        </is>
+      <c r="D14" s="3" t="n">
+        <v>32700</v>
       </c>
       <c r="E14" s="4" t="n">
         <v>1480</v>
       </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Not published on 100 scale</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="n">
+      <c r="F14" s="5" t="n">
         <v>0.24</v>
       </c>
+      <c r="G14" s="6" t="n">
+        <v>25024</v>
+      </c>
       <c r="H14" s="6" t="n">
-        <v>25024</v>
+        <v>5979</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>5979</v>
-      </c>
-      <c r="J14" s="6" t="n">
         <v>850</v>
       </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024 cycle); 2026 cycle data not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="42" customHeight="1">
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>University of Tennessee, Knoxville</t>
@@ -1122,38 +1025,31 @@
       <c r="C15" s="3" t="n">
         <v>52000</v>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Not published for $300k+; overall avg net price ~$22,300 used</t>
-        </is>
+      <c r="D15" s="3" t="n">
+        <v>22300</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>1280</v>
       </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Not published on 100 scale</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="n">
+      <c r="F15" s="5" t="n">
         <v>0.416</v>
       </c>
+      <c r="G15" s="6" t="n">
+        <v>59764</v>
+      </c>
       <c r="H15" s="6" t="n">
-        <v>59764</v>
+        <v>24863</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>24863</v>
-      </c>
-      <c r="J15" s="6" t="n">
         <v>6800</v>
       </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024 cycle); 2026 cycle data not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="42" customHeight="1">
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Virginia Tech</t>
@@ -1167,38 +1063,31 @@
       <c r="C16" s="3" t="n">
         <v>50000</v>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Not published for $300k+; overall avg net price ~$25,800 used</t>
-        </is>
+      <c r="D16" s="3" t="n">
+        <v>25800</v>
       </c>
       <c r="E16" s="4" t="n">
         <v>1360</v>
       </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Not published on 100 scale</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="n">
+      <c r="F16" s="5" t="n">
         <v>0.5478000000000001</v>
       </c>
+      <c r="G16" s="6" t="n">
+        <v>52296</v>
+      </c>
       <c r="H16" s="6" t="n">
-        <v>52296</v>
+        <v>28636</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>28636</v>
-      </c>
-      <c r="J16" s="6" t="n">
         <v>6800</v>
       </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024 cycle); 2026 cycle data not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="42" customHeight="1">
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Wake Forest University</t>
@@ -1212,34 +1101,27 @@
       <c r="C17" s="3" t="n">
         <v>88200</v>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Not published for $300k+; overall avg net price ~$41,900 used</t>
-        </is>
+      <c r="D17" s="3" t="n">
+        <v>41900</v>
       </c>
       <c r="E17" s="4" t="n">
         <v>1470</v>
       </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Not published on 100 scale</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="n">
+      <c r="F17" s="5" t="n">
         <v>0.2167</v>
       </c>
+      <c r="G17" s="6" t="n">
+        <v>18727</v>
+      </c>
       <c r="H17" s="6" t="n">
-        <v>18727</v>
+        <v>4058</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>4058</v>
-      </c>
-      <c r="J17" s="6" t="n">
         <v>1450</v>
       </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024 cycle); 2026 cycle data not yet published.</t>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Early Action deadline column and EA-specific accept rates
- New column: Early Action Deadline. Where a school offers EA, the EA date
  is listed; where it doesn't, the earliest non-binding priority deadline
  is listed and the application type is flagged in Notes.
- Acceptance Rate column now text-formatted to include the school's EA
  acceptance rate in parentheses when the school publishes it; where it
  doesn't, the cell says 'EA rate not published'.
- Miami and Syracuse rows list both EA and ED deadlines.
- Wake Forest flagged: no open EA (ED I/II only; EA is first-gen only).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CUhjAk7h6xF2a3djroFRRG
</commit_message>
<xml_diff>
--- a/college_research.xlsx
+++ b/college_research.xlsx
@@ -16,9 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -65,7 +64,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -77,9 +76,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -450,19 +446,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -493,31 +490,36 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Accept Rate</t>
+          <t>Accept Rate (EA if published)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Early Action Deadline</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Applicants (2026)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Admitted (2026)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Enrolled (2026)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Notes / Cycle Used</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
+    <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Clemson University</t>
@@ -537,25 +539,32 @@
       <c r="E2" s="4" t="n">
         <v>1325</v>
       </c>
-      <c r="F2" s="5" t="n">
-        <v>0.383</v>
-      </c>
-      <c r="G2" s="6" t="n">
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>38.3% (EA rate not published)</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Oct 15 (EA)</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="n">
         <v>61517</v>
       </c>
-      <c r="H2" s="6" t="n">
+      <c r="I2" s="5" t="n">
         <v>23586</v>
       </c>
-      <c r="I2" s="6" t="n">
+      <c r="J2" s="5" t="n">
         <v>4326</v>
       </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="28" customHeight="1">
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Early Action non-binding; materials due Nov 1. 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Florida Atlantic University</t>
@@ -575,25 +584,32 @@
       <c r="E3" s="4" t="n">
         <v>1120</v>
       </c>
-      <c r="F3" s="5" t="n">
-        <v>0.6613</v>
-      </c>
-      <c r="G3" s="6" t="n">
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>66.1%</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Nov 15 (Priority)</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="n">
         <v>31511</v>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="I3" s="5" t="n">
         <v>20838</v>
       </c>
-      <c r="I3" s="6" t="n">
+      <c r="J3" s="5" t="n">
         <v>4900</v>
       </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Rolling admissions (no EA); priority deadline Nov 15. 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Florida State University</t>
@@ -613,25 +629,32 @@
       <c r="E4" s="4" t="n">
         <v>1350</v>
       </c>
-      <c r="F4" s="5" t="n">
-        <v>0.2422</v>
-      </c>
-      <c r="G4" s="6" t="n">
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>24.2%</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Oct 15 (Priority)</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="n">
         <v>78272</v>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="I4" s="5" t="n">
         <v>18954</v>
       </c>
-      <c r="I4" s="6" t="n">
+      <c r="J4" s="5" t="n">
         <v>6800</v>
       </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="28" customHeight="1">
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>No EA; single Nov 1 priority app deadline (Oct 15 for scholarships). 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>NC State University</t>
@@ -651,25 +674,32 @@
       <c r="E5" s="4" t="n">
         <v>1370</v>
       </c>
-      <c r="F5" s="5" t="n">
-        <v>0.417</v>
-      </c>
-      <c r="G5" s="6" t="n">
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>41.7% (EA ~48%)</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Oct 15 (EA)</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="n">
         <v>44043</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="I5" s="5" t="n">
         <v>18381</v>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="J5" s="5" t="n">
         <v>5412</v>
       </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="28" customHeight="1">
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Early Action non-binding. 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Penn State (University Park)</t>
@@ -689,25 +719,32 @@
       <c r="E6" s="4" t="n">
         <v>1330</v>
       </c>
-      <c r="F6" s="5" t="n">
-        <v>0.6056</v>
-      </c>
-      <c r="G6" s="6" t="n">
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>60.6% (EA rate not published)</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Nov 1 (EA)</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="n">
         <v>88478</v>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="I6" s="5" t="n">
         <v>53579</v>
       </c>
-      <c r="I6" s="6" t="n">
+      <c r="J6" s="5" t="n">
         <v>9800</v>
       </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="28" customHeight="1">
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Early Action non-binding (introduced 2023). 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Syracuse University</t>
@@ -727,25 +764,32 @@
       <c r="E7" s="4" t="n">
         <v>1360</v>
       </c>
-      <c r="F7" s="5" t="n">
-        <v>0.4592</v>
-      </c>
-      <c r="G7" s="6" t="n">
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>45.9% (ED: ~60%; EA rate not published)</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Nov 1 (EA &amp; ED I); ED II Jan 5</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="n">
         <v>44480</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="I7" s="5" t="n">
         <v>20427</v>
       </c>
-      <c r="I7" s="6" t="n">
+      <c r="J7" s="5" t="n">
         <v>3835</v>
       </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="28" customHeight="1">
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>University of Alabama</t>
@@ -765,25 +809,32 @@
       <c r="E8" s="4" t="n">
         <v>1290</v>
       </c>
-      <c r="F8" s="5" t="n">
-        <v>0.7659999999999999</v>
-      </c>
-      <c r="G8" s="6" t="n">
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>76.6% (EA rate not published)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Dec 15 (Priority)</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="n">
         <v>56795</v>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="I8" s="5" t="n">
         <v>43531</v>
       </c>
-      <c r="I8" s="6" t="n">
+      <c r="J8" s="5" t="n">
         <v>8039</v>
       </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="28" customHeight="1">
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Rolling admissions (no EA); priority deadline Dec 15. 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>University of Connecticut</t>
@@ -803,25 +854,32 @@
       <c r="E9" s="4" t="n">
         <v>1340</v>
       </c>
-      <c r="F9" s="5" t="n">
-        <v>0.5239</v>
-      </c>
-      <c r="G9" s="6" t="n">
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>52.4% (EA rate not published)</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Nov 1 (EA)</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="n">
         <v>55479</v>
       </c>
-      <c r="H9" s="6" t="n">
+      <c r="I9" s="5" t="n">
         <v>29065</v>
       </c>
-      <c r="I9" s="6" t="n">
+      <c r="J9" s="5" t="n">
         <v>3800</v>
       </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="28" customHeight="1">
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Early Action non-binding. 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>University of Delaware</t>
@@ -841,25 +899,32 @@
       <c r="E10" s="4" t="n">
         <v>1295</v>
       </c>
-      <c r="F10" s="5" t="n">
-        <v>0.706</v>
-      </c>
-      <c r="G10" s="6" t="n">
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>70.6% (EA rate not published)</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Nov 1 (EA)</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="n">
         <v>39995</v>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="I10" s="5" t="n">
         <v>28238</v>
       </c>
-      <c r="I10" s="6" t="n">
+      <c r="J10" s="5" t="n">
         <v>4400</v>
       </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="28" customHeight="1">
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Early Action non-binding. 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>University of Louisville</t>
@@ -879,25 +944,32 @@
       <c r="E11" s="4" t="n">
         <v>1150</v>
       </c>
-      <c r="F11" s="5" t="n">
-        <v>0.7940999999999999</v>
-      </c>
-      <c r="G11" s="6" t="n">
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>79.4%</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Dec 15 (Priority)</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="n">
         <v>15668</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="I11" s="5" t="n">
         <v>12442</v>
       </c>
-      <c r="I11" s="6" t="n">
+      <c r="J11" s="5" t="n">
         <v>2900</v>
       </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="28" customHeight="1">
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Rolling admissions (no EA); priority deadline Dec 15. 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>University of Miami</t>
@@ -917,25 +989,32 @@
       <c r="E12" s="4" t="n">
         <v>1400</v>
       </c>
-      <c r="F12" s="5" t="n">
-        <v>0.189</v>
-      </c>
-      <c r="G12" s="6" t="n">
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>18.9% (ED: 44.3%; EA rate not published)</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Nov 1 (EA &amp; ED I); ED II Jan 5</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="n">
         <v>53954</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="I12" s="5" t="n">
         <v>10195</v>
       </c>
-      <c r="I12" s="6" t="n">
+      <c r="J12" s="5" t="n">
         <v>2400</v>
       </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="28" customHeight="1">
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>University of Pittsburgh</t>
@@ -955,25 +1034,32 @@
       <c r="E13" s="4" t="n">
         <v>1360</v>
       </c>
-      <c r="F13" s="5" t="n">
-        <v>0.5808</v>
-      </c>
-      <c r="G13" s="6" t="n">
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>58.1%</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Dec 1 (Priority)</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="n">
         <v>60898</v>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="I13" s="5" t="n">
         <v>35372</v>
       </c>
-      <c r="I13" s="6" t="n">
+      <c r="J13" s="5" t="n">
         <v>4596</v>
       </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="28" customHeight="1">
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Rolling admissions (no EA); priority deadline Dec 1. 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>University of Richmond</t>
@@ -993,25 +1079,32 @@
       <c r="E14" s="4" t="n">
         <v>1480</v>
       </c>
-      <c r="F14" s="5" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="G14" s="6" t="n">
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>24.0% (EA rate not published)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Nov 1 (EA)</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="n">
         <v>25024</v>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="I14" s="5" t="n">
         <v>5979</v>
       </c>
-      <c r="I14" s="6" t="n">
+      <c r="J14" s="5" t="n">
         <v>850</v>
       </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1">
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>University of Tennessee, Knoxville</t>
@@ -1031,25 +1124,32 @@
       <c r="E15" s="4" t="n">
         <v>1280</v>
       </c>
-      <c r="F15" s="5" t="n">
-        <v>0.416</v>
-      </c>
-      <c r="G15" s="6" t="n">
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>41.6% (EA rate not published)</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Nov 1 (EA)</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="n">
         <v>59764</v>
       </c>
-      <c r="H15" s="6" t="n">
+      <c r="I15" s="5" t="n">
         <v>24863</v>
       </c>
-      <c r="I15" s="6" t="n">
+      <c r="J15" s="5" t="n">
         <v>6800</v>
       </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="28" customHeight="1">
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Early Action non-binding. 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Virginia Tech</t>
@@ -1069,25 +1169,32 @@
       <c r="E16" s="4" t="n">
         <v>1360</v>
       </c>
-      <c r="F16" s="5" t="n">
-        <v>0.5478000000000001</v>
-      </c>
-      <c r="G16" s="6" t="n">
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>54.8% (EA rate not published)</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Dec 1 (EA)</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="n">
         <v>52296</v>
       </c>
-      <c r="H16" s="6" t="n">
+      <c r="I16" s="5" t="n">
         <v>28636</v>
       </c>
-      <c r="I16" s="6" t="n">
+      <c r="J16" s="5" t="n">
         <v>6800</v>
       </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="28" customHeight="1">
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Offers EA (non-binding) plus ED (binding, Nov 1). 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Wake Forest University</t>
@@ -1107,21 +1214,28 @@
       <c r="E17" s="4" t="n">
         <v>1470</v>
       </c>
-      <c r="F17" s="5" t="n">
-        <v>0.2167</v>
-      </c>
-      <c r="G17" s="6" t="n">
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>21.7% (ED I/II admits ~50% of class)</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Nov 15 (ED I; EA is first-gen only)</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="n">
         <v>18727</v>
       </c>
-      <c r="H17" s="6" t="n">
+      <c r="I17" s="5" t="n">
         <v>4058</v>
       </c>
-      <c r="I17" s="6" t="n">
+      <c r="J17" s="5" t="n">
         <v>1450</v>
       </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>2024-25 CDS (fall 2024); 2026 cycle not yet published.</t>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>No open EA — offers ED I (Nov 15) and ED II (Jan 1), both binding; EA restricted to first-generation applicants. 2024-25 CDS.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Swap FSU out; add Boston College and Georgia Tech
- Removed Florida State University from the roster.
- Added Boston College (ED-only, 16.2% overall).
- Added Georgia Tech (two EA rounds, ~14% overall; GA residents 33%).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CUhjAk7h6xF2a3djroFRRG
</commit_message>
<xml_diff>
--- a/college_research.xlsx
+++ b/college_research.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -522,386 +522,386 @@
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Clemson University</t>
+          <t>Boston College</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Clemson, SC</t>
+          <t>Chestnut Hill, MA</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>52206</v>
+        <v>92798</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>25700</v>
+        <v>40800</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>1325</v>
+        <v>1500</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>38.3% (EA rate not published)</t>
+          <t>16.2% (ED: ~33%; no EA)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Oct 15 (EA)</t>
+          <t>Nov 1 (ED I); ED II Jan 1</t>
         </is>
       </c>
       <c r="H2" s="5" t="n">
-        <v>61517</v>
+        <v>36525</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>23586</v>
+        <v>5917</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>4326</v>
+        <v>2400</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Early Action non-binding; materials due Nov 1. 2024-25 CDS.</t>
+          <t>No Early Action; offers ED I (Nov 1) and ED II (Jan 1), both binding. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Florida Atlantic University</t>
+          <t>Clemson University</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Boca Raton, FL</t>
+          <t>Clemson, SC</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>42382</v>
+        <v>52206</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>13600</v>
+        <v>25700</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>1120</v>
+        <v>1325</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>66.1%</t>
+          <t>38.3% (EA rate not published)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Nov 15 (Priority)</t>
+          <t>Oct 15 (EA)</t>
         </is>
       </c>
       <c r="H3" s="5" t="n">
-        <v>31511</v>
+        <v>61517</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>20838</v>
+        <v>23586</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>4900</v>
+        <v>4326</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Rolling admissions (no EA); priority deadline Nov 15. 2024-25 CDS.</t>
+          <t>Early Action non-binding; materials due Nov 1. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Florida State University</t>
+          <t>Florida Atlantic University</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Tallahassee, FL</t>
+          <t>Boca Raton, FL</t>
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>41427</v>
+        <v>42382</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>14600</v>
+        <v>13600</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>1350</v>
+        <v>1120</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>24.2%</t>
+          <t>66.1%</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Oct 15 (Priority)</t>
+          <t>Nov 15 (Priority)</t>
         </is>
       </c>
       <c r="H4" s="5" t="n">
-        <v>78272</v>
+        <v>31511</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>18954</v>
+        <v>20838</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>6800</v>
+        <v>4900</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>No EA; single Nov 1 priority app deadline (Oct 15 for scholarships). 2024-25 CDS.</t>
+          <t>Rolling admissions (no EA); priority deadline Nov 15. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>NC State University</t>
+          <t>Georgia Institute of Technology</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Raleigh, NC</t>
+          <t>Atlanta, GA</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>51285</v>
+        <v>52152</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>16900</v>
+        <v>18500</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>1370</v>
+        <v>1450</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>41.7% (EA ~48%)</t>
+          <t>14% overall (EA GA: 33%, EA non-res: ~13%)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Oct 15 (EA)</t>
+          <t>Oct 15 (EA-1, GA residents); Nov 1 (EA-2, non-residents)</t>
         </is>
       </c>
       <c r="H5" s="5" t="n">
-        <v>44043</v>
+        <v>59712</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>18381</v>
+        <v>8250</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>5412</v>
+        <v>3900</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Early Action non-binding. 2024-25 CDS.</t>
+          <t>Two Early Action rounds (both non-binding); no ED. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Penn State (University Park)</t>
+          <t>NC State University</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>University Park, PA</t>
+          <t>Raleigh, NC</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>63284</v>
+        <v>51285</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>29200</v>
+        <v>16900</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>1330</v>
+        <v>1370</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>60.6% (EA rate not published)</t>
+          <t>41.7% (EA ~48%)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Nov 1 (EA)</t>
+          <t>Oct 15 (EA)</t>
         </is>
       </c>
       <c r="H6" s="5" t="n">
-        <v>88478</v>
+        <v>44043</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>53579</v>
+        <v>18381</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>9800</v>
+        <v>5412</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Early Action non-binding (introduced 2023). 2024-25 CDS.</t>
+          <t>Early Action non-binding. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Syracuse University</t>
+          <t>Penn State (University Park)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Syracuse, NY</t>
+          <t>University Park, PA</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>87840</v>
+        <v>63284</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>48215</v>
+        <v>29200</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>1360</v>
+        <v>1330</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>45.9% (ED: ~60%; EA rate not published)</t>
+          <t>60.6% (EA rate not published)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Nov 1 (EA &amp; ED I); ED II Jan 5</t>
+          <t>Nov 1 (EA)</t>
         </is>
       </c>
       <c r="H7" s="5" t="n">
-        <v>44480</v>
+        <v>88478</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>20427</v>
+        <v>53579</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>3835</v>
+        <v>9800</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
+          <t>Early Action non-binding (introduced 2023). 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>University of Alabama</t>
+          <t>Syracuse University</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Tuscaloosa, AL</t>
+          <t>Syracuse, NY</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>55916</v>
+        <v>87840</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>26900</v>
+        <v>48215</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>1290</v>
+        <v>1360</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>76.6% (EA rate not published)</t>
+          <t>45.9% (ED: ~60%; EA rate not published)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Dec 15 (Priority)</t>
+          <t>Nov 1 (EA &amp; ED I); ED II Jan 5</t>
         </is>
       </c>
       <c r="H8" s="5" t="n">
-        <v>56795</v>
+        <v>44480</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>43531</v>
+        <v>20427</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>8039</v>
+        <v>3835</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Rolling admissions (no EA); priority deadline Dec 15. 2024-25 CDS.</t>
+          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>University of Connecticut</t>
+          <t>University of Alabama</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Storrs, CT</t>
+          <t>Tuscaloosa, AL</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>58780</v>
+        <v>55916</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>23800</v>
+        <v>26900</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>1340</v>
+        <v>1290</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>52.4% (EA rate not published)</t>
+          <t>76.6% (EA rate not published)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Nov 1 (EA)</t>
+          <t>Dec 15 (Priority)</t>
         </is>
       </c>
       <c r="H9" s="5" t="n">
-        <v>55479</v>
+        <v>56795</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>29065</v>
+        <v>43531</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>3800</v>
+        <v>8039</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Early Action non-binding. 2024-25 CDS.</t>
+          <t>Rolling admissions (no EA); priority deadline Dec 15. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>University of Delaware</t>
+          <t>University of Connecticut</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Newark, DE</t>
+          <t>Storrs, CT</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>56090</v>
+        <v>58780</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>24500</v>
+        <v>23800</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>1295</v>
+        <v>1340</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>70.6% (EA rate not published)</t>
+          <t>52.4% (EA rate not published)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -910,13 +910,13 @@
         </is>
       </c>
       <c r="H10" s="5" t="n">
-        <v>39995</v>
+        <v>55479</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>28238</v>
+        <v>29065</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>4400</v>
+        <v>3800</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -927,206 +927,206 @@
     <row r="11" ht="34" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>University of Louisville</t>
+          <t>University of Delaware</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Louisville, KY</t>
+          <t>Newark, DE</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>44500</v>
+        <v>56090</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>19785</v>
+        <v>24500</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>1150</v>
+        <v>1295</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>79.4%</t>
+          <t>70.6% (EA rate not published)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Dec 15 (Priority)</t>
+          <t>Nov 1 (EA)</t>
         </is>
       </c>
       <c r="H11" s="5" t="n">
-        <v>15668</v>
+        <v>39995</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>12442</v>
+        <v>28238</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>2900</v>
+        <v>4400</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Rolling admissions (no EA); priority deadline Dec 15. 2024-25 CDS.</t>
+          <t>Early Action non-binding. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>University of Miami</t>
+          <t>University of Louisville</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Coral Gables, FL</t>
+          <t>Louisville, KY</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>93892</v>
+        <v>44500</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>44600</v>
+        <v>19785</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>1400</v>
+        <v>1150</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>18.9% (ED: 44.3%; EA rate not published)</t>
+          <t>79.4%</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Nov 1 (EA &amp; ED I); ED II Jan 5</t>
+          <t>Dec 15 (Priority)</t>
         </is>
       </c>
       <c r="H12" s="5" t="n">
-        <v>53954</v>
+        <v>15668</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>10195</v>
+        <v>12442</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>2400</v>
+        <v>2900</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
+          <t>Rolling admissions (no EA); priority deadline Dec 15. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>University of Pittsburgh</t>
+          <t>University of Miami</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Coral Gables, FL</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>60310</v>
+        <v>93892</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>27400</v>
+        <v>44600</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>1360</v>
+        <v>1400</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>58.1%</t>
+          <t>18.9% (ED: 44.3%; EA rate not published)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Dec 1 (Priority)</t>
+          <t>Nov 1 (EA &amp; ED I); ED II Jan 5</t>
         </is>
       </c>
       <c r="H13" s="5" t="n">
-        <v>60898</v>
+        <v>53954</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>35372</v>
+        <v>10195</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>4596</v>
+        <v>2400</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Rolling admissions (no EA); priority deadline Dec 1. 2024-25 CDS.</t>
+          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="34" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>University of Richmond</t>
+          <t>University of Pittsburgh</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>84930</v>
+        <v>60310</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>32700</v>
+        <v>27400</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>1480</v>
+        <v>1360</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>24.0% (EA rate not published)</t>
+          <t>58.1%</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Nov 1 (EA)</t>
+          <t>Dec 1 (Priority)</t>
         </is>
       </c>
       <c r="H14" s="5" t="n">
-        <v>25024</v>
+        <v>60898</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>5979</v>
+        <v>35372</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>850</v>
+        <v>4596</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
+          <t>Rolling admissions (no EA); priority deadline Dec 1. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="34" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>University of Tennessee, Knoxville</t>
+          <t>University of Richmond</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Knoxville, TN</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>52000</v>
+        <v>84930</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>22300</v>
+        <v>32700</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>1280</v>
+        <v>1480</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>41.6% (EA rate not published)</t>
+          <t>24.0% (EA rate not published)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1135,105 +1135,150 @@
         </is>
       </c>
       <c r="H15" s="5" t="n">
-        <v>59764</v>
+        <v>25024</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>24863</v>
+        <v>5979</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>6800</v>
+        <v>850</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Early Action non-binding. 2024-25 CDS.</t>
+          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="34" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Virginia Tech</t>
+          <t>University of Tennessee, Knoxville</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Blacksburg, VA</t>
+          <t>Knoxville, TN</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>50000</v>
+        <v>52000</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>25800</v>
+        <v>22300</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>1360</v>
+        <v>1280</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>54.8% (EA rate not published)</t>
+          <t>41.6% (EA rate not published)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Dec 1 (EA)</t>
+          <t>Nov 1 (EA)</t>
         </is>
       </c>
       <c r="H16" s="5" t="n">
-        <v>52296</v>
+        <v>59764</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>28636</v>
+        <v>24863</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>6800</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Offers EA (non-binding) plus ED (binding, Nov 1). 2024-25 CDS.</t>
+          <t>Early Action non-binding. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="34" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>Virginia Tech</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Blacksburg, VA</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>25800</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>1360</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>54.8% (EA rate not published)</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Dec 1 (EA)</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>52296</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>28636</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>6800</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Offers EA (non-binding) plus ED (binding, Nov 1). 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>Wake Forest University</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Winston-Salem, NC</t>
         </is>
       </c>
-      <c r="C17" s="3" t="n">
+      <c r="C18" s="3" t="n">
         <v>88200</v>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D18" s="3" t="n">
         <v>41900</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E18" s="4" t="n">
         <v>1470</v>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>21.7% (ED I/II admits ~50% of class)</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Nov 15 (ED I; EA is first-gen only)</t>
         </is>
       </c>
-      <c r="H17" s="5" t="n">
+      <c r="H18" s="5" t="n">
         <v>18727</v>
       </c>
-      <c r="I17" s="5" t="n">
+      <c r="I18" s="5" t="n">
         <v>4058</v>
       </c>
-      <c r="J17" s="5" t="n">
+      <c r="J18" s="5" t="n">
         <v>1450</v>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>No open EA — offers ED I (Nov 15) and ED II (Jan 1), both binding; EA restricted to first-generation applicants. 2024-25 CDS.</t>
         </is>

</xml_diff>

<commit_message>
Add Michigan State University to the roster
MSU (East Lansing, MI): 84.8% overall accept rate, SAT median 1260,
OOS COA 2,632, EA deadline Nov 1 (non-binding).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CUhjAk7h6xF2a3djroFRRG
</commit_message>
<xml_diff>
--- a/college_research.xlsx
+++ b/college_research.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -702,41 +702,41 @@
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>NC State University</t>
+          <t>Michigan State University</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Raleigh, NC</t>
+          <t>East Lansing, MI</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>51285</v>
+        <v>62632</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>16900</v>
+        <v>21200</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>1370</v>
+        <v>1260</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>41.7% (EA ~48%)</t>
+          <t>84.8% (EA rate not published)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Oct 15 (EA)</t>
+          <t>Nov 1 (EA)</t>
         </is>
       </c>
       <c r="H6" s="5" t="n">
-        <v>44043</v>
+        <v>62138</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>18381</v>
+        <v>52690</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>5412</v>
+        <v>9649</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
@@ -747,206 +747,206 @@
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Penn State (University Park)</t>
+          <t>NC State University</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>University Park, PA</t>
+          <t>Raleigh, NC</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>63284</v>
+        <v>51285</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>29200</v>
+        <v>16900</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>1330</v>
+        <v>1370</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>60.6% (EA rate not published)</t>
+          <t>41.7% (EA ~48%)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Nov 1 (EA)</t>
+          <t>Oct 15 (EA)</t>
         </is>
       </c>
       <c r="H7" s="5" t="n">
-        <v>88478</v>
+        <v>44043</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>53579</v>
+        <v>18381</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>9800</v>
+        <v>5412</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Early Action non-binding (introduced 2023). 2024-25 CDS.</t>
+          <t>Early Action non-binding. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Syracuse University</t>
+          <t>Penn State (University Park)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Syracuse, NY</t>
+          <t>University Park, PA</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>87840</v>
+        <v>63284</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>48215</v>
+        <v>29200</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>1360</v>
+        <v>1330</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>45.9% (ED: ~60%; EA rate not published)</t>
+          <t>60.6% (EA rate not published)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Nov 1 (EA &amp; ED I); ED II Jan 5</t>
+          <t>Nov 1 (EA)</t>
         </is>
       </c>
       <c r="H8" s="5" t="n">
-        <v>44480</v>
+        <v>88478</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>20427</v>
+        <v>53579</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>3835</v>
+        <v>9800</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
+          <t>Early Action non-binding (introduced 2023). 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>University of Alabama</t>
+          <t>Syracuse University</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Tuscaloosa, AL</t>
+          <t>Syracuse, NY</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>55916</v>
+        <v>87840</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>26900</v>
+        <v>48215</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>1290</v>
+        <v>1360</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>76.6% (EA rate not published)</t>
+          <t>45.9% (ED: ~60%; EA rate not published)</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Dec 15 (Priority)</t>
+          <t>Nov 1 (EA &amp; ED I); ED II Jan 5</t>
         </is>
       </c>
       <c r="H9" s="5" t="n">
-        <v>56795</v>
+        <v>44480</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>43531</v>
+        <v>20427</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>8039</v>
+        <v>3835</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Rolling admissions (no EA); priority deadline Dec 15. 2024-25 CDS.</t>
+          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>University of Connecticut</t>
+          <t>University of Alabama</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Storrs, CT</t>
+          <t>Tuscaloosa, AL</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>58780</v>
+        <v>55916</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>23800</v>
+        <v>26900</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>1340</v>
+        <v>1290</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>52.4% (EA rate not published)</t>
+          <t>76.6% (EA rate not published)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Nov 1 (EA)</t>
+          <t>Dec 15 (Priority)</t>
         </is>
       </c>
       <c r="H10" s="5" t="n">
-        <v>55479</v>
+        <v>56795</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>29065</v>
+        <v>43531</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>3800</v>
+        <v>8039</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Early Action non-binding. 2024-25 CDS.</t>
+          <t>Rolling admissions (no EA); priority deadline Dec 15. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="34" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>University of Delaware</t>
+          <t>University of Connecticut</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Newark, DE</t>
+          <t>Storrs, CT</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>56090</v>
+        <v>58780</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>24500</v>
+        <v>23800</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>1295</v>
+        <v>1340</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>70.6% (EA rate not published)</t>
+          <t>52.4% (EA rate not published)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -955,13 +955,13 @@
         </is>
       </c>
       <c r="H11" s="5" t="n">
-        <v>39995</v>
+        <v>55479</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>28238</v>
+        <v>29065</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>4400</v>
+        <v>3800</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
@@ -972,206 +972,206 @@
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>University of Louisville</t>
+          <t>University of Delaware</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Louisville, KY</t>
+          <t>Newark, DE</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>44500</v>
+        <v>56090</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>19785</v>
+        <v>24500</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>1150</v>
+        <v>1295</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>79.4%</t>
+          <t>70.6% (EA rate not published)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Dec 15 (Priority)</t>
+          <t>Nov 1 (EA)</t>
         </is>
       </c>
       <c r="H12" s="5" t="n">
-        <v>15668</v>
+        <v>39995</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>12442</v>
+        <v>28238</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>2900</v>
+        <v>4400</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Rolling admissions (no EA); priority deadline Dec 15. 2024-25 CDS.</t>
+          <t>Early Action non-binding. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>University of Miami</t>
+          <t>University of Louisville</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Coral Gables, FL</t>
+          <t>Louisville, KY</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>93892</v>
+        <v>44500</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>44600</v>
+        <v>19785</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>1400</v>
+        <v>1150</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>18.9% (ED: 44.3%; EA rate not published)</t>
+          <t>79.4%</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Nov 1 (EA &amp; ED I); ED II Jan 5</t>
+          <t>Dec 15 (Priority)</t>
         </is>
       </c>
       <c r="H13" s="5" t="n">
-        <v>53954</v>
+        <v>15668</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>10195</v>
+        <v>12442</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>2400</v>
+        <v>2900</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
+          <t>Rolling admissions (no EA); priority deadline Dec 15. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="34" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>University of Pittsburgh</t>
+          <t>University of Miami</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Pittsburgh, PA</t>
+          <t>Coral Gables, FL</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>60310</v>
+        <v>93892</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>27400</v>
+        <v>44600</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>1360</v>
+        <v>1400</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>58.1%</t>
+          <t>18.9% (ED: 44.3%; EA rate not published)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Dec 1 (Priority)</t>
+          <t>Nov 1 (EA &amp; ED I); ED II Jan 5</t>
         </is>
       </c>
       <c r="H14" s="5" t="n">
-        <v>60898</v>
+        <v>53954</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>35372</v>
+        <v>10195</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>4596</v>
+        <v>2400</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Rolling admissions (no EA); priority deadline Dec 1. 2024-25 CDS.</t>
+          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="34" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>University of Richmond</t>
+          <t>University of Pittsburgh</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Pittsburgh, PA</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>84930</v>
+        <v>60310</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>32700</v>
+        <v>27400</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>1480</v>
+        <v>1360</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>24.0% (EA rate not published)</t>
+          <t>58.1%</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Nov 1 (EA)</t>
+          <t>Dec 1 (Priority)</t>
         </is>
       </c>
       <c r="H15" s="5" t="n">
-        <v>25024</v>
+        <v>60898</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>5979</v>
+        <v>35372</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>850</v>
+        <v>4596</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
+          <t>Rolling admissions (no EA); priority deadline Dec 1. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="34" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>University of Tennessee, Knoxville</t>
+          <t>University of Richmond</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Knoxville, TN</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>52000</v>
+        <v>84930</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>22300</v>
+        <v>32700</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>1280</v>
+        <v>1480</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>41.6% (EA rate not published)</t>
+          <t>24.0% (EA rate not published)</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1180,105 +1180,150 @@
         </is>
       </c>
       <c r="H16" s="5" t="n">
-        <v>59764</v>
+        <v>25024</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>24863</v>
+        <v>5979</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>6800</v>
+        <v>850</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Early Action non-binding. 2024-25 CDS.</t>
+          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="34" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Virginia Tech</t>
+          <t>University of Tennessee, Knoxville</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Blacksburg, VA</t>
+          <t>Knoxville, TN</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>50000</v>
+        <v>52000</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>25800</v>
+        <v>22300</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>1360</v>
+        <v>1280</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>54.8% (EA rate not published)</t>
+          <t>41.6% (EA rate not published)</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Dec 1 (EA)</t>
+          <t>Nov 1 (EA)</t>
         </is>
       </c>
       <c r="H17" s="5" t="n">
-        <v>52296</v>
+        <v>59764</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>28636</v>
+        <v>24863</v>
       </c>
       <c r="J17" s="5" t="n">
         <v>6800</v>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Offers EA (non-binding) plus ED (binding, Nov 1). 2024-25 CDS.</t>
+          <t>Early Action non-binding. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="34" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>Virginia Tech</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Blacksburg, VA</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>25800</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>1360</v>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>54.8% (EA rate not published)</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Dec 1 (EA)</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>52296</v>
+      </c>
+      <c r="I18" s="5" t="n">
+        <v>28636</v>
+      </c>
+      <c r="J18" s="5" t="n">
+        <v>6800</v>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Offers EA (non-binding) plus ED (binding, Nov 1). 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>Wake Forest University</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Winston-Salem, NC</t>
         </is>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="C19" s="3" t="n">
         <v>88200</v>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D19" s="3" t="n">
         <v>41900</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="E19" s="4" t="n">
         <v>1470</v>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>21.7% (ED I/II admits ~50% of class)</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Nov 15 (ED I; EA is first-gen only)</t>
         </is>
       </c>
-      <c r="H18" s="5" t="n">
+      <c r="H19" s="5" t="n">
         <v>18727</v>
       </c>
-      <c r="I18" s="5" t="n">
+      <c r="I19" s="5" t="n">
         <v>4058</v>
       </c>
-      <c r="J18" s="5" t="n">
+      <c r="J19" s="5" t="n">
         <v>1450</v>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>No open EA — offers ED I (Nov 15) and ED II (Jan 1), both binding; EA restricted to first-generation applicants. 2024-25 CDS.</t>
         </is>

</xml_diff>

<commit_message>
Add OOS accept rate, public/private, and supplemental-essay columns
- New column 'OOS Accept Rate' next to Accept Rate — in-state for UConn per
  request; N/A for privates; noted where residency-specific rate isn't
  officially published.
- New column 'Public / Private' just before Notes.
- New column 'Supplemental Essays' with parenthesized count when present.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CUhjAk7h6xF2a3djroFRRG
</commit_message>
<xml_diff>
--- a/college_research.xlsx
+++ b/college_research.xlsx
@@ -446,23 +446,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42" customHeight="1">
+    <row r="1" ht="44" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>School</t>
@@ -495,31 +498,46 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>OOS Accept Rate (In-State for UConn)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Early Action Deadline</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Applicants (2026)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Admitted (2026)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Enrolled (2026)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Supplemental Essays</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Public / Private</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Notes / Cycle Used</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="34" customHeight="1">
+    <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Boston College</t>
@@ -546,25 +564,40 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>N/A (private — no state split)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>Nov 1 (ED I); ED II Jan 1</t>
         </is>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="I2" s="5" t="n">
         <v>36525</v>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="J2" s="5" t="n">
         <v>5917</v>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="K2" s="5" t="n">
         <v>2400</v>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>No Early Action; offers ED I (Nov 1) and ED II (Jan 1), both binding. 2024-25 CDS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="34" customHeight="1">
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Yes (1)</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>No EA; ED I (Nov 1) and ED II (Jan 1), both binding. 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="36" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Clemson University</t>
@@ -591,25 +624,40 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
+          <t>~35%</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
           <t>Oct 15 (EA)</t>
         </is>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="I3" s="5" t="n">
         <v>61517</v>
       </c>
-      <c r="I3" s="5" t="n">
+      <c r="J3" s="5" t="n">
         <v>23586</v>
       </c>
-      <c r="J3" s="5" t="n">
+      <c r="K3" s="5" t="n">
         <v>4326</v>
       </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Early Action non-binding; materials due Nov 1. 2024-25 CDS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="34" customHeight="1">
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Optional (1)</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>EA non-binding; materials due Nov 1. 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Florida Atlantic University</t>
@@ -636,25 +684,40 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
+          <t>OOS rate not published separately</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
           <t>Nov 15 (Priority)</t>
         </is>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="I4" s="5" t="n">
         <v>31511</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="J4" s="5" t="n">
         <v>20838</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="K4" s="5" t="n">
         <v>4900</v>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>Rolling admissions (no EA); priority deadline Nov 15. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="34" customHeight="1">
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Georgia Institute of Technology</t>
@@ -681,25 +744,40 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
+          <t>~10%</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
           <t>Oct 15 (EA-1, GA residents); Nov 1 (EA-2, non-residents)</t>
         </is>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="I5" s="5" t="n">
         <v>59712</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="J5" s="5" t="n">
         <v>8250</v>
       </c>
-      <c r="J5" s="5" t="n">
+      <c r="K5" s="5" t="n">
         <v>3900</v>
       </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>Two Early Action rounds (both non-binding); no ED. 2024-25 CDS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Yes (1) — reduced from 3 for 2026-27</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Two EA rounds (both non-binding); no ED. 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Michigan State University</t>
@@ -726,25 +804,40 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
+          <t>OOS rate not published separately (~80%+ est.)</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
           <t>Nov 1 (EA)</t>
         </is>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="I6" s="5" t="n">
         <v>62138</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="J6" s="5" t="n">
         <v>52690</v>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="K6" s="5" t="n">
         <v>9649</v>
       </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>Early Action non-binding. 2024-25 CDS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>No (personal statement optional)</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>EA non-binding. 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>NC State University</t>
@@ -771,25 +864,40 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
+          <t>~34%</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
           <t>Oct 15 (EA)</t>
         </is>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="I7" s="5" t="n">
         <v>44043</v>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="J7" s="5" t="n">
         <v>18381</v>
       </c>
-      <c r="J7" s="5" t="n">
+      <c r="K7" s="5" t="n">
         <v>5412</v>
       </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>Early Action non-binding. 2024-25 CDS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Yes (3)</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>EA non-binding. 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Penn State (University Park)</t>
@@ -816,25 +924,40 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
+          <t>~55-60%</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
           <t>Nov 1 (EA)</t>
         </is>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="I8" s="5" t="n">
         <v>88478</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="J8" s="5" t="n">
         <v>53579</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="K8" s="5" t="n">
         <v>9800</v>
       </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Early Action non-binding (introduced 2023). 2024-25 CDS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1">
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Yes (1) — personal statement</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>EA non-binding (introduced 2023). 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="36" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Syracuse University</t>
@@ -861,25 +984,40 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
+          <t>N/A (private — no state split)</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
           <t>Nov 1 (EA &amp; ED I); ED II Jan 5</t>
         </is>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="I9" s="5" t="n">
         <v>44480</v>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="J9" s="5" t="n">
         <v>20427</v>
       </c>
-      <c r="J9" s="5" t="n">
+      <c r="K9" s="5" t="n">
         <v>3835</v>
       </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Yes (1)</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>EA plus ED I and ED II (binding). 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>University of Alabama</t>
@@ -906,25 +1044,40 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
+          <t>OOS rate not published separately (~76% est.)</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
           <t>Dec 15 (Priority)</t>
         </is>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="I10" s="5" t="n">
         <v>56795</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="J10" s="5" t="n">
         <v>43531</v>
       </c>
-      <c r="J10" s="5" t="n">
+      <c r="K10" s="5" t="n">
         <v>8039</v>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>Rolling admissions (no EA); priority deadline Dec 15. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="34" customHeight="1">
+    <row r="11" ht="36" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>University of Connecticut</t>
@@ -951,25 +1104,40 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
+          <t>In-state: ~54%</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
           <t>Nov 1 (EA)</t>
         </is>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="I11" s="5" t="n">
         <v>55479</v>
       </c>
-      <c r="I11" s="5" t="n">
+      <c r="J11" s="5" t="n">
         <v>29065</v>
       </c>
-      <c r="J11" s="5" t="n">
+      <c r="K11" s="5" t="n">
         <v>3800</v>
       </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>Early Action non-binding. 2024-25 CDS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1">
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Yes (1) — short answer</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>EA non-binding. UConn in-state acceptance shown per user request. 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="36" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>University of Delaware</t>
@@ -996,25 +1164,40 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
+          <t>~70% (similar to overall)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
           <t>Nov 1 (EA)</t>
         </is>
       </c>
-      <c r="H12" s="5" t="n">
+      <c r="I12" s="5" t="n">
         <v>39995</v>
       </c>
-      <c r="I12" s="5" t="n">
+      <c r="J12" s="5" t="n">
         <v>28238</v>
       </c>
-      <c r="J12" s="5" t="n">
+      <c r="K12" s="5" t="n">
         <v>4400</v>
       </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Early Action non-binding. 2024-25 CDS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>No (essay optional)</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>EA non-binding. 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>University of Louisville</t>
@@ -1041,25 +1224,40 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
+          <t>OOS rate not published separately</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
           <t>Dec 15 (Priority)</t>
         </is>
       </c>
-      <c r="H13" s="5" t="n">
+      <c r="I13" s="5" t="n">
         <v>15668</v>
       </c>
-      <c r="I13" s="5" t="n">
+      <c r="J13" s="5" t="n">
         <v>12442</v>
       </c>
-      <c r="J13" s="5" t="n">
+      <c r="K13" s="5" t="n">
         <v>2900</v>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>Rolling admissions (no EA); priority deadline Dec 15. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="34" customHeight="1">
+    <row r="14" ht="36" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>University of Miami</t>
@@ -1086,25 +1284,40 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
+          <t>N/A (private — no state split)</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
           <t>Nov 1 (EA &amp; ED I); ED II Jan 5</t>
         </is>
       </c>
-      <c r="H14" s="5" t="n">
+      <c r="I14" s="5" t="n">
         <v>53954</v>
       </c>
-      <c r="I14" s="5" t="n">
+      <c r="J14" s="5" t="n">
         <v>10195</v>
       </c>
-      <c r="J14" s="5" t="n">
+      <c r="K14" s="5" t="n">
         <v>2400</v>
       </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="34" customHeight="1">
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Yes (1) — dropped from 2 for 2026-27</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>EA plus ED I and ED II (binding). 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>University of Pittsburgh</t>
@@ -1131,25 +1344,40 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
+          <t>~50%</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
           <t>Dec 1 (Priority)</t>
         </is>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="I15" s="5" t="n">
         <v>60898</v>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="J15" s="5" t="n">
         <v>35372</v>
       </c>
-      <c r="J15" s="5" t="n">
+      <c r="K15" s="5" t="n">
         <v>4596</v>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>No (essay optional)</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>Rolling admissions (no EA); priority deadline Dec 1. 2024-25 CDS.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="34" customHeight="1">
+    <row r="16" ht="36" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>University of Richmond</t>
@@ -1176,25 +1404,40 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
+          <t>N/A (private — no state split)</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
           <t>Nov 1 (EA)</t>
         </is>
       </c>
-      <c r="H16" s="5" t="n">
+      <c r="I16" s="5" t="n">
         <v>25024</v>
       </c>
-      <c r="I16" s="5" t="n">
+      <c r="J16" s="5" t="n">
         <v>5979</v>
       </c>
-      <c r="J16" s="5" t="n">
+      <c r="K16" s="5" t="n">
         <v>850</v>
       </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Offers EA (non-binding) plus ED I and ED II (binding). 2024-25 CDS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="34" customHeight="1">
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Yes (3)</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>EA plus ED I and ED II (binding). 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>University of Tennessee, Knoxville</t>
@@ -1221,25 +1464,40 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
+          <t>~40-45%</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
           <t>Nov 1 (EA)</t>
         </is>
       </c>
-      <c r="H17" s="5" t="n">
+      <c r="I17" s="5" t="n">
         <v>59764</v>
       </c>
-      <c r="I17" s="5" t="n">
+      <c r="J17" s="5" t="n">
         <v>24863</v>
       </c>
-      <c r="J17" s="5" t="n">
+      <c r="K17" s="5" t="n">
         <v>6800</v>
       </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Early Action non-binding. 2024-25 CDS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="34" customHeight="1">
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>EA non-binding. 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="36" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Virginia Tech</t>
@@ -1266,25 +1524,40 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
+          <t>~58.7%</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
           <t>Dec 1 (EA)</t>
         </is>
       </c>
-      <c r="H18" s="5" t="n">
+      <c r="I18" s="5" t="n">
         <v>52296</v>
       </c>
-      <c r="I18" s="5" t="n">
+      <c r="J18" s="5" t="n">
         <v>28636</v>
       </c>
-      <c r="J18" s="5" t="n">
+      <c r="K18" s="5" t="n">
         <v>6800</v>
       </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Offers EA (non-binding) plus ED (binding, Nov 1). 2024-25 CDS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="34" customHeight="1">
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Yes (4) — Ut Prosim short-answer prompts</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>EA plus ED (binding, Nov 1). 2024-25 CDS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Wake Forest University</t>
@@ -1311,21 +1584,36 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
+          <t>N/A (private — no state split)</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
           <t>Nov 15 (ED I; EA is first-gen only)</t>
         </is>
       </c>
-      <c r="H19" s="5" t="n">
+      <c r="I19" s="5" t="n">
         <v>18727</v>
       </c>
-      <c r="I19" s="5" t="n">
+      <c r="J19" s="5" t="n">
         <v>4058</v>
       </c>
-      <c r="J19" s="5" t="n">
+      <c r="K19" s="5" t="n">
         <v>1450</v>
       </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>No open EA — offers ED I (Nov 15) and ED II (Jan 1), both binding; EA restricted to first-generation applicants. 2024-25 CDS.</t>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Yes (5) — trimmed to 1 for 2026-27 with recommendation added</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Private</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>No open EA; ED I (Nov 15) and ED II (Jan 1) binding; EA first-gen only. 2024-25 CDS.</t>
         </is>
       </c>
     </row>

</xml_diff>